<commit_message>
IST-Zeiten für heutige Termin im Arbeitsplan ergänzt
</commit_message>
<xml_diff>
--- a/docs/inprogress/Arbeitsplan.xlsx
+++ b/docs/inprogress/Arbeitsplan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1-PCTower\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1-PCTower\Documents\GitHub\306_top_down_shooter\docs\inprogress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{506238F5-2BF6-4493-A2A8-8E8C0FB2FD63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4970373D-30CB-4A18-A6D4-25C1887F89DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2763,7 +2763,7 @@
       <c r="M5" s="131"/>
       <c r="N5" s="130">
         <f>SUM(N10:Q10,N12:Q12,N14:Q14,N16:Q16,N18:Q18,N20:Q20,N24:Q24,N26:Q26,N28:Q28,N30:Q30,N32:Q32,N36:Q36,N40:Q40,N42:Q42,N44:Q44,N46:Q46,N48:Q48,N50:Q50,N52:Q52,N54:Q54,N58:Q58,N60:Q60,N62:Q62,N64:Q64,N66:Q66,N68:Q68,N70:Q70,N72:Q72,N76:Q76,N78:Q78,N80:Q80,N82:Q82,N86:Q86,N88:Q88,N90:Q90,N92:Q92,N96:Q96,N98:Q98,N102:Q102,N106:Q106,N34:Q34)</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="O5" s="131"/>
       <c r="P5" s="131"/>
@@ -2842,7 +2842,7 @@
       <c r="M6" s="140"/>
       <c r="N6" s="138">
         <f t="shared" ref="N6" si="1">N4-N5</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="O6" s="139"/>
       <c r="P6" s="139"/>
@@ -5054,7 +5054,7 @@
       <c r="D40" s="43"/>
       <c r="E40" s="44">
         <f>SUM(F40:BA40)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F40" s="7"/>
       <c r="G40" s="5"/>
@@ -5064,10 +5064,18 @@
       <c r="K40" s="5"/>
       <c r="L40" s="5"/>
       <c r="M40" s="6"/>
-      <c r="N40" s="106"/>
-      <c r="O40" s="107"/>
-      <c r="P40" s="107"/>
-      <c r="Q40" s="108"/>
+      <c r="N40" s="106">
+        <v>1</v>
+      </c>
+      <c r="O40" s="107">
+        <v>1</v>
+      </c>
+      <c r="P40" s="107">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="108">
+        <v>0</v>
+      </c>
       <c r="R40" s="106"/>
       <c r="S40" s="107"/>
       <c r="T40" s="107"/>
@@ -5186,7 +5194,7 @@
       <c r="D42" s="43"/>
       <c r="E42" s="44">
         <f>SUM(F42:BA42)</f>
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="F42" s="7"/>
       <c r="G42" s="5"/>
@@ -5196,10 +5204,18 @@
       <c r="K42" s="5"/>
       <c r="L42" s="5"/>
       <c r="M42" s="6"/>
-      <c r="N42" s="106"/>
-      <c r="O42" s="107"/>
-      <c r="P42" s="107"/>
-      <c r="Q42" s="108"/>
+      <c r="N42" s="106">
+        <v>1</v>
+      </c>
+      <c r="O42" s="107">
+        <v>0.25</v>
+      </c>
+      <c r="P42" s="107">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="108">
+        <v>0</v>
+      </c>
       <c r="R42" s="106"/>
       <c r="S42" s="107"/>
       <c r="T42" s="107"/>
@@ -5318,7 +5334,7 @@
       <c r="D44" s="43"/>
       <c r="E44" s="44">
         <f>SUM(F44:BA44)</f>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="F44" s="7"/>
       <c r="G44" s="5"/>
@@ -5328,10 +5344,18 @@
       <c r="K44" s="5"/>
       <c r="L44" s="5"/>
       <c r="M44" s="6"/>
-      <c r="N44" s="106"/>
-      <c r="O44" s="107"/>
-      <c r="P44" s="107"/>
-      <c r="Q44" s="108"/>
+      <c r="N44" s="106">
+        <v>0.2</v>
+      </c>
+      <c r="O44" s="107">
+        <v>0</v>
+      </c>
+      <c r="P44" s="107">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="108">
+        <v>0</v>
+      </c>
       <c r="R44" s="106"/>
       <c r="S44" s="107"/>
       <c r="T44" s="107"/>
@@ -5450,7 +5474,7 @@
       <c r="D46" s="43"/>
       <c r="E46" s="44">
         <f>SUM(F46:BA46)</f>
-        <v>0</v>
+        <v>1.55</v>
       </c>
       <c r="F46" s="7"/>
       <c r="G46" s="5"/>
@@ -5460,10 +5484,18 @@
       <c r="K46" s="5"/>
       <c r="L46" s="5"/>
       <c r="M46" s="6"/>
-      <c r="N46" s="106"/>
-      <c r="O46" s="107"/>
-      <c r="P46" s="107"/>
-      <c r="Q46" s="108"/>
+      <c r="N46" s="106">
+        <v>0.3</v>
+      </c>
+      <c r="O46" s="107">
+        <v>0.25</v>
+      </c>
+      <c r="P46" s="107">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="108">
+        <v>1</v>
+      </c>
       <c r="R46" s="106"/>
       <c r="S46" s="107"/>
       <c r="T46" s="107"/>
@@ -5582,7 +5614,7 @@
       <c r="D48" s="43"/>
       <c r="E48" s="44">
         <f>SUM(F48:BA48)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F48" s="7"/>
       <c r="G48" s="5"/>
@@ -5592,10 +5624,18 @@
       <c r="K48" s="5"/>
       <c r="L48" s="5"/>
       <c r="M48" s="6"/>
-      <c r="N48" s="106"/>
-      <c r="O48" s="107"/>
-      <c r="P48" s="107"/>
-      <c r="Q48" s="108"/>
+      <c r="N48" s="106">
+        <v>1</v>
+      </c>
+      <c r="O48" s="107">
+        <v>1</v>
+      </c>
+      <c r="P48" s="107">
+        <v>1</v>
+      </c>
+      <c r="Q48" s="108">
+        <v>0</v>
+      </c>
       <c r="R48" s="106"/>
       <c r="S48" s="107"/>
       <c r="T48" s="107"/>
@@ -5714,7 +5754,7 @@
       <c r="D50" s="43"/>
       <c r="E50" s="44">
         <f>SUM(F50:BA50)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F50" s="7"/>
       <c r="G50" s="5"/>
@@ -5724,10 +5764,18 @@
       <c r="K50" s="5"/>
       <c r="L50" s="5"/>
       <c r="M50" s="6"/>
-      <c r="N50" s="106"/>
-      <c r="O50" s="107"/>
-      <c r="P50" s="107"/>
-      <c r="Q50" s="108"/>
+      <c r="N50" s="106">
+        <v>1</v>
+      </c>
+      <c r="O50" s="107">
+        <v>1</v>
+      </c>
+      <c r="P50" s="107">
+        <v>1</v>
+      </c>
+      <c r="Q50" s="108">
+        <v>1</v>
+      </c>
       <c r="R50" s="106"/>
       <c r="S50" s="107"/>
       <c r="T50" s="107"/>
@@ -5846,7 +5894,7 @@
       <c r="D52" s="43"/>
       <c r="E52" s="44">
         <f>SUM(F52:BA52)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F52" s="7"/>
       <c r="G52" s="5"/>
@@ -5856,10 +5904,18 @@
       <c r="K52" s="5"/>
       <c r="L52" s="5"/>
       <c r="M52" s="6"/>
-      <c r="N52" s="106"/>
-      <c r="O52" s="107"/>
-      <c r="P52" s="107"/>
-      <c r="Q52" s="108"/>
+      <c r="N52" s="106">
+        <v>0.5</v>
+      </c>
+      <c r="O52" s="107">
+        <v>0.5</v>
+      </c>
+      <c r="P52" s="107">
+        <v>0.5</v>
+      </c>
+      <c r="Q52" s="108">
+        <v>0.5</v>
+      </c>
       <c r="R52" s="106"/>
       <c r="S52" s="107"/>
       <c r="T52" s="107"/>
@@ -9013,7 +9069,7 @@
       <c r="BH105" s="58"/>
       <c r="BI105" s="55">
         <f>SUM(E9:E106)</f>
-        <v>28.75</v>
+        <v>42.75</v>
       </c>
       <c r="BJ105" s="57" t="s">
         <v>11</v>
@@ -9095,7 +9151,7 @@
       </c>
       <c r="E107" s="61">
         <f>SUM(E9:E106)</f>
-        <v>28.75</v>
+        <v>42.75</v>
       </c>
       <c r="BB107" s="29"/>
       <c r="BC107" s="29"/>
@@ -9106,7 +9162,7 @@
       <c r="BG107" s="121"/>
       <c r="BH107" s="151">
         <f>IF((BH104-BI105)&gt;0,(BH104-BI105),(BH104-BI105)*(1))</f>
-        <v>55.25</v>
+        <v>41.25</v>
       </c>
       <c r="BI107" s="152"/>
       <c r="BJ107" s="57" t="s">
@@ -9299,7 +9355,7 @@
       <c r="BD110" s="67"/>
       <c r="BF110" s="145">
         <f>IF((BH107)&lt;=0,(BH107/24)*(-1),BH107/24)</f>
-        <v>2.3020833333333335</v>
+        <v>1.71875</v>
       </c>
       <c r="BG110" s="145"/>
       <c r="BH110" s="145"/>

</xml_diff>

<commit_message>
Update Arbeitsplan - 20.03.2026
</commit_message>
<xml_diff>
--- a/docs/inprogress/Arbeitsplan.xlsx
+++ b/docs/inprogress/Arbeitsplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1-PCTower\Documents\GitHub\306_top_down_shooter\docs\inprogress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4970373D-30CB-4A18-A6D4-25C1887F89DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4AB14E1-2BDF-49AD-BA3A-18242931FE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="585" yWindow="315" windowWidth="24060" windowHeight="12825" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1095,9 +1095,75 @@
     <xf numFmtId="2" fontId="2" fillId="15" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="7" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="1" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1131,74 +1197,8 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="7" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="6" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="6" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="6" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2468,59 +2468,59 @@
   <sheetData>
     <row r="1" spans="2:57" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B1" s="19"/>
-      <c r="C1" s="137" t="s">
+      <c r="C1" s="133" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="137"/>
-      <c r="E1" s="137"/>
-      <c r="F1" s="137"/>
-      <c r="G1" s="137"/>
-      <c r="H1" s="137"/>
-      <c r="I1" s="137"/>
-      <c r="J1" s="137"/>
-      <c r="K1" s="137"/>
-      <c r="L1" s="137"/>
-      <c r="M1" s="137"/>
-      <c r="N1" s="137"/>
-      <c r="O1" s="137"/>
-      <c r="P1" s="137"/>
-      <c r="Q1" s="137"/>
-      <c r="R1" s="137"/>
-      <c r="S1" s="137"/>
-      <c r="T1" s="137"/>
-      <c r="U1" s="137"/>
-      <c r="V1" s="137"/>
-      <c r="W1" s="137"/>
-      <c r="X1" s="137"/>
-      <c r="Y1" s="137"/>
-      <c r="Z1" s="137"/>
-      <c r="AA1" s="137"/>
-      <c r="AB1" s="137"/>
-      <c r="AC1" s="137"/>
-      <c r="AD1" s="137"/>
-      <c r="AE1" s="137"/>
-      <c r="AF1" s="137"/>
-      <c r="AG1" s="137"/>
-      <c r="AH1" s="137"/>
-      <c r="AI1" s="137"/>
-      <c r="AJ1" s="137"/>
-      <c r="AK1" s="137"/>
-      <c r="AL1" s="137"/>
-      <c r="AM1" s="137"/>
-      <c r="AN1" s="137"/>
-      <c r="AO1" s="137"/>
-      <c r="AP1" s="137"/>
-      <c r="AQ1" s="137"/>
-      <c r="AR1" s="137"/>
-      <c r="AS1" s="137"/>
-      <c r="AT1" s="137"/>
-      <c r="AU1" s="137"/>
-      <c r="AV1" s="137"/>
-      <c r="AW1" s="137"/>
-      <c r="AX1" s="137"/>
-      <c r="AY1" s="137"/>
-      <c r="AZ1" s="137"/>
-      <c r="BA1" s="137"/>
+      <c r="D1" s="133"/>
+      <c r="E1" s="133"/>
+      <c r="F1" s="133"/>
+      <c r="G1" s="133"/>
+      <c r="H1" s="133"/>
+      <c r="I1" s="133"/>
+      <c r="J1" s="133"/>
+      <c r="K1" s="133"/>
+      <c r="L1" s="133"/>
+      <c r="M1" s="133"/>
+      <c r="N1" s="133"/>
+      <c r="O1" s="133"/>
+      <c r="P1" s="133"/>
+      <c r="Q1" s="133"/>
+      <c r="R1" s="133"/>
+      <c r="S1" s="133"/>
+      <c r="T1" s="133"/>
+      <c r="U1" s="133"/>
+      <c r="V1" s="133"/>
+      <c r="W1" s="133"/>
+      <c r="X1" s="133"/>
+      <c r="Y1" s="133"/>
+      <c r="Z1" s="133"/>
+      <c r="AA1" s="133"/>
+      <c r="AB1" s="133"/>
+      <c r="AC1" s="133"/>
+      <c r="AD1" s="133"/>
+      <c r="AE1" s="133"/>
+      <c r="AF1" s="133"/>
+      <c r="AG1" s="133"/>
+      <c r="AH1" s="133"/>
+      <c r="AI1" s="133"/>
+      <c r="AJ1" s="133"/>
+      <c r="AK1" s="133"/>
+      <c r="AL1" s="133"/>
+      <c r="AM1" s="133"/>
+      <c r="AN1" s="133"/>
+      <c r="AO1" s="133"/>
+      <c r="AP1" s="133"/>
+      <c r="AQ1" s="133"/>
+      <c r="AR1" s="133"/>
+      <c r="AS1" s="133"/>
+      <c r="AT1" s="133"/>
+      <c r="AU1" s="133"/>
+      <c r="AV1" s="133"/>
+      <c r="AW1" s="133"/>
+      <c r="AX1" s="133"/>
+      <c r="AY1" s="133"/>
+      <c r="AZ1" s="133"/>
+      <c r="BA1" s="133"/>
       <c r="BB1" s="20"/>
       <c r="BC1" s="20"/>
       <c r="BD1" s="20"/>
@@ -2530,66 +2530,66 @@
       <c r="C2" s="23"/>
       <c r="D2" s="24"/>
       <c r="E2" s="25"/>
-      <c r="F2" s="118" t="s">
+      <c r="F2" s="130" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="118"/>
-      <c r="H2" s="118"/>
-      <c r="I2" s="118"/>
-      <c r="J2" s="118" t="s">
+      <c r="G2" s="130"/>
+      <c r="H2" s="130"/>
+      <c r="I2" s="130"/>
+      <c r="J2" s="130" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="118"/>
-      <c r="L2" s="118"/>
-      <c r="M2" s="118"/>
-      <c r="N2" s="118" t="s">
+      <c r="K2" s="130"/>
+      <c r="L2" s="130"/>
+      <c r="M2" s="130"/>
+      <c r="N2" s="130" t="s">
         <v>15</v>
       </c>
-      <c r="O2" s="118"/>
-      <c r="P2" s="118"/>
-      <c r="Q2" s="118"/>
-      <c r="R2" s="118" t="s">
+      <c r="O2" s="130"/>
+      <c r="P2" s="130"/>
+      <c r="Q2" s="130"/>
+      <c r="R2" s="130" t="s">
         <v>16</v>
       </c>
-      <c r="S2" s="118"/>
-      <c r="T2" s="118"/>
-      <c r="U2" s="118"/>
-      <c r="V2" s="118" t="s">
+      <c r="S2" s="130"/>
+      <c r="T2" s="130"/>
+      <c r="U2" s="130"/>
+      <c r="V2" s="130" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="118"/>
-      <c r="X2" s="118"/>
-      <c r="Y2" s="118"/>
-      <c r="Z2" s="118" t="s">
+      <c r="W2" s="130"/>
+      <c r="X2" s="130"/>
+      <c r="Y2" s="130"/>
+      <c r="Z2" s="130" t="s">
         <v>18</v>
       </c>
-      <c r="AA2" s="118"/>
-      <c r="AB2" s="118"/>
-      <c r="AC2" s="118"/>
-      <c r="AD2" s="118"/>
-      <c r="AE2" s="118"/>
-      <c r="AF2" s="118"/>
-      <c r="AG2" s="118"/>
-      <c r="AH2" s="118"/>
-      <c r="AI2" s="118"/>
-      <c r="AJ2" s="118"/>
-      <c r="AK2" s="118"/>
-      <c r="AL2" s="134"/>
-      <c r="AM2" s="134"/>
-      <c r="AN2" s="134"/>
-      <c r="AO2" s="134"/>
-      <c r="AP2" s="142"/>
-      <c r="AQ2" s="141"/>
-      <c r="AR2" s="141"/>
-      <c r="AS2" s="141"/>
-      <c r="AT2" s="118"/>
-      <c r="AU2" s="118"/>
-      <c r="AV2" s="118"/>
-      <c r="AW2" s="118"/>
-      <c r="AX2" s="141"/>
-      <c r="AY2" s="141"/>
-      <c r="AZ2" s="141"/>
-      <c r="BA2" s="141"/>
+      <c r="AA2" s="130"/>
+      <c r="AB2" s="130"/>
+      <c r="AC2" s="130"/>
+      <c r="AD2" s="130"/>
+      <c r="AE2" s="130"/>
+      <c r="AF2" s="130"/>
+      <c r="AG2" s="130"/>
+      <c r="AH2" s="130"/>
+      <c r="AI2" s="130"/>
+      <c r="AJ2" s="130"/>
+      <c r="AK2" s="130"/>
+      <c r="AL2" s="152"/>
+      <c r="AM2" s="152"/>
+      <c r="AN2" s="152"/>
+      <c r="AO2" s="152"/>
+      <c r="AP2" s="138"/>
+      <c r="AQ2" s="137"/>
+      <c r="AR2" s="137"/>
+      <c r="AS2" s="137"/>
+      <c r="AT2" s="130"/>
+      <c r="AU2" s="130"/>
+      <c r="AV2" s="130"/>
+      <c r="AW2" s="130"/>
+      <c r="AX2" s="137"/>
+      <c r="AY2" s="137"/>
+      <c r="AZ2" s="137"/>
+      <c r="BA2" s="137"/>
       <c r="BB2" s="26"/>
       <c r="BC2" s="26"/>
       <c r="BE2" s="85"/>
@@ -2599,220 +2599,220 @@
       <c r="C3" s="23"/>
       <c r="D3" s="24"/>
       <c r="E3" s="25"/>
-      <c r="F3" s="135">
+      <c r="F3" s="122">
         <v>46084</v>
       </c>
-      <c r="G3" s="136"/>
-      <c r="H3" s="136"/>
-      <c r="I3" s="136"/>
-      <c r="J3" s="135">
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="122">
         <v>46091</v>
       </c>
-      <c r="K3" s="136"/>
-      <c r="L3" s="136"/>
-      <c r="M3" s="136"/>
-      <c r="N3" s="135">
+      <c r="K3" s="123"/>
+      <c r="L3" s="123"/>
+      <c r="M3" s="123"/>
+      <c r="N3" s="122">
         <v>46098</v>
       </c>
-      <c r="O3" s="136"/>
-      <c r="P3" s="136"/>
-      <c r="Q3" s="136"/>
-      <c r="R3" s="135">
+      <c r="O3" s="123"/>
+      <c r="P3" s="123"/>
+      <c r="Q3" s="123"/>
+      <c r="R3" s="122">
         <v>46099</v>
       </c>
-      <c r="S3" s="136"/>
-      <c r="T3" s="136"/>
-      <c r="U3" s="136"/>
-      <c r="V3" s="135">
+      <c r="S3" s="123"/>
+      <c r="T3" s="123"/>
+      <c r="U3" s="123"/>
+      <c r="V3" s="122">
         <v>46100</v>
       </c>
-      <c r="W3" s="136"/>
-      <c r="X3" s="136"/>
-      <c r="Y3" s="136"/>
-      <c r="Z3" s="135">
+      <c r="W3" s="123"/>
+      <c r="X3" s="123"/>
+      <c r="Y3" s="123"/>
+      <c r="Z3" s="122">
         <v>41053</v>
       </c>
-      <c r="AA3" s="136"/>
-      <c r="AB3" s="136"/>
-      <c r="AC3" s="136"/>
-      <c r="AD3" s="135"/>
-      <c r="AE3" s="136"/>
-      <c r="AF3" s="136"/>
-      <c r="AG3" s="136"/>
-      <c r="AH3" s="135"/>
-      <c r="AI3" s="136"/>
-      <c r="AJ3" s="136"/>
-      <c r="AK3" s="136"/>
-      <c r="AL3" s="135"/>
-      <c r="AM3" s="136"/>
-      <c r="AN3" s="136"/>
-      <c r="AO3" s="136"/>
-      <c r="AP3" s="135"/>
-      <c r="AQ3" s="136"/>
-      <c r="AR3" s="136"/>
-      <c r="AS3" s="136"/>
-      <c r="AT3" s="135"/>
-      <c r="AU3" s="136"/>
-      <c r="AV3" s="136"/>
-      <c r="AW3" s="136"/>
-      <c r="AX3" s="135"/>
-      <c r="AY3" s="136"/>
-      <c r="AZ3" s="136"/>
-      <c r="BA3" s="136"/>
+      <c r="AA3" s="123"/>
+      <c r="AB3" s="123"/>
+      <c r="AC3" s="123"/>
+      <c r="AD3" s="122"/>
+      <c r="AE3" s="123"/>
+      <c r="AF3" s="123"/>
+      <c r="AG3" s="123"/>
+      <c r="AH3" s="122"/>
+      <c r="AI3" s="123"/>
+      <c r="AJ3" s="123"/>
+      <c r="AK3" s="123"/>
+      <c r="AL3" s="122"/>
+      <c r="AM3" s="123"/>
+      <c r="AN3" s="123"/>
+      <c r="AO3" s="123"/>
+      <c r="AP3" s="122"/>
+      <c r="AQ3" s="123"/>
+      <c r="AR3" s="123"/>
+      <c r="AS3" s="123"/>
+      <c r="AT3" s="122"/>
+      <c r="AU3" s="123"/>
+      <c r="AV3" s="123"/>
+      <c r="AW3" s="123"/>
+      <c r="AX3" s="122"/>
+      <c r="AY3" s="123"/>
+      <c r="AZ3" s="123"/>
+      <c r="BA3" s="123"/>
       <c r="BB3" s="29"/>
       <c r="BC3" s="29"/>
       <c r="BE3" s="86"/>
     </row>
     <row r="4" spans="2:57" s="27" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="28"/>
-      <c r="C4" s="143" t="s">
+      <c r="C4" s="139" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="143"/>
-      <c r="E4" s="144"/>
-      <c r="F4" s="132">
+      <c r="D4" s="139"/>
+      <c r="E4" s="140"/>
+      <c r="F4" s="127">
         <f>SUM(F9:I9,F11:I11,F13:I13,F15:I15,F17:I17,F19:I19,F23:I23,F25:I25,F27:I27,F29:I29,F31:I31,F33:I33,F39:I39,F41:I41,F43:I43,F45:I45,F47:I47,F49:I49,F51:I51,F53:I53,F57:I57,F59:I59,F61:I61,F63:I63,F65:I65,F67:I67,F69:I69,F71:I71,F75:I75,F77:I77,F79:I79,F81:I81,F85:I85,F87:I87,F89:I89,F91:I91,F95:I95,F97:I97,F101:I101,F105:I105,F35:I35)</f>
         <v>14</v>
       </c>
-      <c r="G4" s="133"/>
-      <c r="H4" s="133"/>
-      <c r="I4" s="133"/>
-      <c r="J4" s="132">
+      <c r="G4" s="128"/>
+      <c r="H4" s="128"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="127">
         <f>SUM(J9:M9,J11:M11,J13:M13,J15:M15,J17:M17,J19:M19,J23:M23,J25:M25,J27:M27,J29:M29,J31:M31,J33:M33,J39:M39,J41:M41,J43:M43,J45:M45,J47:M47,J49:M49,J51:M51,J53:M53,J57:M57,J59:M59,J61:M61,J63:M63,J65:M65,J67:M67,J69:M69,J71:M71,J75:M75,J77:M77,J79:M79,J81:M81,J85:M85,J87:M87,J89:M89,J91:M91,J95:M95,J97:M97,J101:M101,J105:M105,J35:M35)</f>
         <v>14</v>
       </c>
-      <c r="K4" s="133"/>
-      <c r="L4" s="133"/>
-      <c r="M4" s="133"/>
-      <c r="N4" s="132">
+      <c r="K4" s="128"/>
+      <c r="L4" s="128"/>
+      <c r="M4" s="128"/>
+      <c r="N4" s="127">
         <f>SUM(N9:Q9,N11:Q11,N13:Q13,N15:Q15,N17:Q17,N19:Q19,N23:Q23,N25:Q25,N27:Q27,N29:Q29,N31:Q31,N33:Q33,N39:Q39,N41:Q41,N43:Q43,N45:Q45,N47:Q47,N49:Q49,N51:Q51,N53:Q53,N57:Q57,N59:Q59,N61:Q61,N63:Q63,N65:Q65,N67:Q67,N69:Q69,N71:Q71,N75:Q75,N77:Q77,N79:Q79,N81:Q81,N85:Q85,N87:Q87,N89:Q89,N91:Q91,N95:Q95,N97:Q97,N101:Q101,N105:Q105,N35:Q35)</f>
         <v>14</v>
       </c>
-      <c r="O4" s="133"/>
-      <c r="P4" s="133"/>
-      <c r="Q4" s="133"/>
-      <c r="R4" s="132">
+      <c r="O4" s="128"/>
+      <c r="P4" s="128"/>
+      <c r="Q4" s="128"/>
+      <c r="R4" s="127">
         <f>SUM(R9:U9,R11:U11,R13:U13,R15:U15,R17:U17,R19:U19,R23:U23,R25:U25,R27:U27,R29:U29,R31:U31,R33:U33,R39:U39,R41:U41,R43:U43,R45:U45,R47:U47,R49:U49,R51:U51,R53:U53,R57:U57,R59:U59,R61:U61,R63:U63,R65:U65,R67:U67,R69:U69,R71:U71,R75:U75,R77:U77,R79:U79,R81:U81,R85:U85,R87:U87,R89:U89,R91:U91,R95:U95,R97:U97,R101:U101,R105:U105,R35:U35)</f>
         <v>14</v>
       </c>
-      <c r="S4" s="133"/>
-      <c r="T4" s="133"/>
-      <c r="U4" s="133"/>
-      <c r="V4" s="132">
+      <c r="S4" s="128"/>
+      <c r="T4" s="128"/>
+      <c r="U4" s="128"/>
+      <c r="V4" s="127">
         <f>SUM(V9:Y9,V11:Y11,V13:Y13,V15:Y15,V17:Y17,V19:Y19,V23:Y23,V25:Y25,V27:Y27,V29:Y29,V31:Y31,V33:Y33,V39:Y39,V41:Y41,V43:Y43,V45:Y45,V47:Y47,V49:Y49,V51:Y51,V53:Y53,V57:Y57,V59:Y59,V61:Y61,V63:Y63,V65:Y65,V67:Y67,V69:Y69,V71:Y71,V75:Y75,V77:Y77,V79:Y79,V81:Y81,V85:Y85,V87:Y87,V89:Y89,V91:Y91,V95:Y95,V97:Y97,V101:Y101,V105:Y105,V35:Y35)</f>
         <v>13.999999999999996</v>
       </c>
-      <c r="W4" s="133"/>
-      <c r="X4" s="133"/>
-      <c r="Y4" s="133"/>
-      <c r="Z4" s="132">
+      <c r="W4" s="128"/>
+      <c r="X4" s="128"/>
+      <c r="Y4" s="128"/>
+      <c r="Z4" s="127">
         <f>SUM(Z9:AC9,Z11:AC11,Z13:AC13,Z15:AC15,Z17:AC17,Z19:AC19,Z23:AC23,Z25:AC25,Z27:AC27,Z29:AC29,Z31:AC31,Z33:AC33,Z39:AC39,Z41:AC41,Z43:AC43,Z45:AC45,Z47:AC47,Z49:AC49,Z51:AC51,Z53:AC53,Z57:AC57,Z59:AC59,Z61:AC61,Z63:AC63,Z65:AC65,Z67:AC67,Z69:AC69,Z71:AC71,Z75:AC75,Z77:AC77,Z79:AC79,Z81:AC81,Z85:AC85,Z87:AC87,Z89:AC89,Z91:AC91,Z95:AC95,Z97:AC97,Z101:AC101,Z105:AC105,Z35:AC35)</f>
         <v>14</v>
       </c>
-      <c r="AA4" s="133"/>
-      <c r="AB4" s="133"/>
-      <c r="AC4" s="133"/>
-      <c r="AD4" s="132"/>
-      <c r="AE4" s="133"/>
-      <c r="AF4" s="133"/>
-      <c r="AG4" s="133"/>
-      <c r="AH4" s="132"/>
-      <c r="AI4" s="133"/>
-      <c r="AJ4" s="133"/>
-      <c r="AK4" s="133"/>
-      <c r="AL4" s="132"/>
-      <c r="AM4" s="133"/>
-      <c r="AN4" s="133"/>
-      <c r="AO4" s="133"/>
-      <c r="AP4" s="132"/>
-      <c r="AQ4" s="133"/>
-      <c r="AR4" s="133"/>
-      <c r="AS4" s="133"/>
-      <c r="AT4" s="132"/>
-      <c r="AU4" s="133"/>
-      <c r="AV4" s="133"/>
-      <c r="AW4" s="133"/>
-      <c r="AX4" s="132"/>
-      <c r="AY4" s="133"/>
-      <c r="AZ4" s="133"/>
-      <c r="BA4" s="133"/>
+      <c r="AA4" s="128"/>
+      <c r="AB4" s="128"/>
+      <c r="AC4" s="128"/>
+      <c r="AD4" s="127"/>
+      <c r="AE4" s="128"/>
+      <c r="AF4" s="128"/>
+      <c r="AG4" s="128"/>
+      <c r="AH4" s="127"/>
+      <c r="AI4" s="128"/>
+      <c r="AJ4" s="128"/>
+      <c r="AK4" s="128"/>
+      <c r="AL4" s="127"/>
+      <c r="AM4" s="128"/>
+      <c r="AN4" s="128"/>
+      <c r="AO4" s="128"/>
+      <c r="AP4" s="127"/>
+      <c r="AQ4" s="128"/>
+      <c r="AR4" s="128"/>
+      <c r="AS4" s="128"/>
+      <c r="AT4" s="127"/>
+      <c r="AU4" s="128"/>
+      <c r="AV4" s="128"/>
+      <c r="AW4" s="128"/>
+      <c r="AX4" s="127"/>
+      <c r="AY4" s="128"/>
+      <c r="AZ4" s="128"/>
+      <c r="BA4" s="128"/>
       <c r="BB4" s="30"/>
       <c r="BC4" s="29"/>
       <c r="BE4" s="86"/>
     </row>
     <row r="5" spans="2:57" s="27" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="28"/>
-      <c r="C5" s="143" t="s">
+      <c r="C5" s="139" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="143"/>
-      <c r="E5" s="144"/>
-      <c r="F5" s="130">
+      <c r="D5" s="139"/>
+      <c r="E5" s="140"/>
+      <c r="F5" s="118">
         <f>SUM(F10:I10,F12:I12,F14:I14,F16:I16,F18:I18,F20:I20,F24:I24,F26:I26,F28:I28,F30:I30,F32:I32,F36:I36,F40:I40,F42:I42,F44:I44,F46:I46,F48:I48,F50:I50,F52:I52,F54:I54,F58:I58,F60:I60,F62:I62,F64:I64,F66:I66,F68:I68,F70:I70,F72:I72,F76:I76,F78:I78,F80:I80,F82:I82,F86:I86,F88:I88,F90:I90,F92:I92,F96:I96,F98:I98,F102:I102,F106:I106,F34:I34)</f>
         <v>14</v>
       </c>
-      <c r="G5" s="131"/>
-      <c r="H5" s="131"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="130">
+      <c r="G5" s="119"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="119"/>
+      <c r="J5" s="118">
         <f>SUM(J10:M10,J12:M12,J14:M14,J16:M16,J18:M18,J20:M20,J24:M24,J26:M26,J28:M28,J30:M30,J32:M32,J36:M36,J40:M40,J42:M42,J44:M44,J46:M46,J48:M48,J50:M50,J52:M52,J54:M54,J58:M58,J60:M60,J62:M62,J64:M64,J66:M66,J68:M68,J70:M70,J72:M72,J76:M76,J78:M78,J80:M80,J82:M82,J86:M86,J88:M88,J90:M90,J92:M92,J96:M96,J98:M98,J102:M102,J106:M106,J34:M34)</f>
         <v>14.75</v>
       </c>
-      <c r="K5" s="131"/>
-      <c r="L5" s="131"/>
-      <c r="M5" s="131"/>
-      <c r="N5" s="130">
+      <c r="K5" s="119"/>
+      <c r="L5" s="119"/>
+      <c r="M5" s="119"/>
+      <c r="N5" s="118">
         <f>SUM(N10:Q10,N12:Q12,N14:Q14,N16:Q16,N18:Q18,N20:Q20,N24:Q24,N26:Q26,N28:Q28,N30:Q30,N32:Q32,N36:Q36,N40:Q40,N42:Q42,N44:Q44,N46:Q46,N48:Q48,N50:Q50,N52:Q52,N54:Q54,N58:Q58,N60:Q60,N62:Q62,N64:Q64,N66:Q66,N68:Q68,N70:Q70,N72:Q72,N76:Q76,N78:Q78,N80:Q80,N82:Q82,N86:Q86,N88:Q88,N90:Q90,N92:Q92,N96:Q96,N98:Q98,N102:Q102,N106:Q106,N34:Q34)</f>
         <v>14</v>
       </c>
-      <c r="O5" s="131"/>
-      <c r="P5" s="131"/>
-      <c r="Q5" s="131"/>
-      <c r="R5" s="130">
+      <c r="O5" s="119"/>
+      <c r="P5" s="119"/>
+      <c r="Q5" s="119"/>
+      <c r="R5" s="118">
         <f>SUM(R10:U10,R12:U12,R14:U14,R16:U16,R18:U18,R20:U20,R24:U24,R26:U26,R28:U28,R30:U30,R32:U32,R36:U36,R40:U40,R42:U42,R44:U44,R46:U46,R48:U48,R50:U50,R52:U52,R54:U54,R58:U58,R60:U60,R62:U62,R64:U64,R66:U66,R68:U68,R70:U70,R72:U72,R76:U76,R78:U78,R80:U80,R82:U82,R86:U86,R88:U88,R90:U90,R92:U92,R96:U96,R98:U98,R102:U102,R106:U106,R34:U34)</f>
-        <v>0</v>
-      </c>
-      <c r="S5" s="131"/>
-      <c r="T5" s="131"/>
-      <c r="U5" s="131"/>
-      <c r="V5" s="130">
+        <v>14</v>
+      </c>
+      <c r="S5" s="119"/>
+      <c r="T5" s="119"/>
+      <c r="U5" s="119"/>
+      <c r="V5" s="118">
         <f>SUM(V10:Y10,V12:Y12,V14:Y14,V16:Y16,V18:Y18,V20:Y20,V24:Y24,V26:Y26,V28:Y28,V30:Y30,V32:Y32,V36:Y36,V40:Y40,V42:Y42,V44:Y44,V46:Y46,V48:Y48,V50:Y50,V52:Y52,V54:Y54,V58:Y58,V60:Y60,V62:Y62,V64:Y64,V66:Y66,V68:Y68,V70:Y70,V72:Y72,V76:Y76,V78:Y78,V80:Y80,V82:Y82,V86:Y86,V88:Y88,V90:Y90,V92:Y92,V96:Y96,V98:Y98,V102:Y102,V106:Y106,V34:Y34)</f>
-        <v>0</v>
-      </c>
-      <c r="W5" s="131"/>
-      <c r="X5" s="131"/>
-      <c r="Y5" s="131"/>
-      <c r="Z5" s="130">
+        <v>13.999999999999996</v>
+      </c>
+      <c r="W5" s="119"/>
+      <c r="X5" s="119"/>
+      <c r="Y5" s="119"/>
+      <c r="Z5" s="118">
         <f>SUM(Z10:AC10,Z12:AC12,Z14:AC14,Z16:AC16,Z18:AC18,Z20:AC20,Z24:AC24,Z26:AC26,Z28:AC28,Z30:AC30,Z32:AC32,Z36:AC36,Z40:AC40,Z42:AC42,Z44:AC44,Z46:AC46,Z48:AC48,Z50:AC50,Z52:AC52,Z54:AC54,Z58:AC58,Z60:AC60,Z62:AC62,Z64:AC64,Z66:AC66,Z68:AC68,Z70:AC70,Z72:AC72,Z76:AC76,Z78:AC78,Z80:AC80,Z82:AC82,Z86:AC86,Z88:AC88,Z90:AC90,Z92:AC92,Z96:AC96,Z98:AC98,Z102:AC102,Z106:AC106,Z34:AC34)</f>
         <v>0</v>
       </c>
-      <c r="AA5" s="131"/>
-      <c r="AB5" s="131"/>
-      <c r="AC5" s="131"/>
-      <c r="AD5" s="130"/>
-      <c r="AE5" s="131"/>
-      <c r="AF5" s="131"/>
-      <c r="AG5" s="131"/>
-      <c r="AH5" s="130"/>
-      <c r="AI5" s="131"/>
-      <c r="AJ5" s="131"/>
-      <c r="AK5" s="131"/>
-      <c r="AL5" s="130"/>
-      <c r="AM5" s="131"/>
-      <c r="AN5" s="131"/>
-      <c r="AO5" s="131"/>
-      <c r="AP5" s="130"/>
-      <c r="AQ5" s="131"/>
-      <c r="AR5" s="131"/>
-      <c r="AS5" s="131"/>
-      <c r="AT5" s="130"/>
-      <c r="AU5" s="131"/>
-      <c r="AV5" s="131"/>
-      <c r="AW5" s="131"/>
-      <c r="AX5" s="130"/>
-      <c r="AY5" s="131"/>
-      <c r="AZ5" s="131"/>
-      <c r="BA5" s="131"/>
+      <c r="AA5" s="119"/>
+      <c r="AB5" s="119"/>
+      <c r="AC5" s="119"/>
+      <c r="AD5" s="118"/>
+      <c r="AE5" s="119"/>
+      <c r="AF5" s="119"/>
+      <c r="AG5" s="119"/>
+      <c r="AH5" s="118"/>
+      <c r="AI5" s="119"/>
+      <c r="AJ5" s="119"/>
+      <c r="AK5" s="119"/>
+      <c r="AL5" s="118"/>
+      <c r="AM5" s="119"/>
+      <c r="AN5" s="119"/>
+      <c r="AO5" s="119"/>
+      <c r="AP5" s="118"/>
+      <c r="AQ5" s="119"/>
+      <c r="AR5" s="119"/>
+      <c r="AS5" s="119"/>
+      <c r="AT5" s="118"/>
+      <c r="AU5" s="119"/>
+      <c r="AV5" s="119"/>
+      <c r="AW5" s="119"/>
+      <c r="AX5" s="118"/>
+      <c r="AY5" s="119"/>
+      <c r="AZ5" s="119"/>
+      <c r="BA5" s="119"/>
       <c r="BB5" s="30"/>
       <c r="BC5" s="29"/>
       <c r="BE5" s="86"/>
@@ -2822,76 +2822,76 @@
       <c r="C6" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="122" t="s">
+      <c r="D6" s="144" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="123"/>
-      <c r="F6" s="138">
+      <c r="E6" s="145"/>
+      <c r="F6" s="134">
         <f>F4-F5</f>
         <v>0</v>
       </c>
-      <c r="G6" s="139"/>
-      <c r="H6" s="139"/>
-      <c r="I6" s="140"/>
-      <c r="J6" s="138">
+      <c r="G6" s="135"/>
+      <c r="H6" s="135"/>
+      <c r="I6" s="136"/>
+      <c r="J6" s="134">
         <f t="shared" ref="J6" si="0">J4-J5</f>
         <v>-0.75</v>
       </c>
-      <c r="K6" s="139"/>
-      <c r="L6" s="139"/>
-      <c r="M6" s="140"/>
-      <c r="N6" s="138">
+      <c r="K6" s="135"/>
+      <c r="L6" s="135"/>
+      <c r="M6" s="136"/>
+      <c r="N6" s="134">
         <f t="shared" ref="N6" si="1">N4-N5</f>
         <v>0</v>
       </c>
-      <c r="O6" s="139"/>
-      <c r="P6" s="139"/>
-      <c r="Q6" s="139"/>
-      <c r="R6" s="138">
+      <c r="O6" s="135"/>
+      <c r="P6" s="135"/>
+      <c r="Q6" s="135"/>
+      <c r="R6" s="134">
         <f t="shared" ref="R6" si="2">R4-R5</f>
-        <v>14</v>
-      </c>
-      <c r="S6" s="139"/>
-      <c r="T6" s="139"/>
-      <c r="U6" s="139"/>
-      <c r="V6" s="138">
+        <v>0</v>
+      </c>
+      <c r="S6" s="135"/>
+      <c r="T6" s="135"/>
+      <c r="U6" s="135"/>
+      <c r="V6" s="134">
         <f t="shared" ref="V6" si="3">V4-V5</f>
-        <v>13.999999999999996</v>
-      </c>
-      <c r="W6" s="139"/>
-      <c r="X6" s="139"/>
-      <c r="Y6" s="139"/>
-      <c r="Z6" s="138">
+        <v>0</v>
+      </c>
+      <c r="W6" s="135"/>
+      <c r="X6" s="135"/>
+      <c r="Y6" s="135"/>
+      <c r="Z6" s="134">
         <f t="shared" ref="Z6" si="4">Z4-Z5</f>
         <v>14</v>
       </c>
-      <c r="AA6" s="139"/>
-      <c r="AB6" s="139"/>
-      <c r="AC6" s="139"/>
-      <c r="AD6" s="138"/>
-      <c r="AE6" s="139"/>
-      <c r="AF6" s="139"/>
-      <c r="AG6" s="139"/>
-      <c r="AH6" s="138"/>
-      <c r="AI6" s="139"/>
-      <c r="AJ6" s="139"/>
-      <c r="AK6" s="139"/>
-      <c r="AL6" s="138"/>
-      <c r="AM6" s="139"/>
-      <c r="AN6" s="139"/>
-      <c r="AO6" s="139"/>
-      <c r="AP6" s="138"/>
-      <c r="AQ6" s="139"/>
-      <c r="AR6" s="139"/>
-      <c r="AS6" s="139"/>
-      <c r="AT6" s="138"/>
-      <c r="AU6" s="139"/>
-      <c r="AV6" s="139"/>
-      <c r="AW6" s="139"/>
-      <c r="AX6" s="138"/>
-      <c r="AY6" s="139"/>
-      <c r="AZ6" s="139"/>
-      <c r="BA6" s="139"/>
+      <c r="AA6" s="135"/>
+      <c r="AB6" s="135"/>
+      <c r="AC6" s="135"/>
+      <c r="AD6" s="134"/>
+      <c r="AE6" s="135"/>
+      <c r="AF6" s="135"/>
+      <c r="AG6" s="135"/>
+      <c r="AH6" s="134"/>
+      <c r="AI6" s="135"/>
+      <c r="AJ6" s="135"/>
+      <c r="AK6" s="135"/>
+      <c r="AL6" s="134"/>
+      <c r="AM6" s="135"/>
+      <c r="AN6" s="135"/>
+      <c r="AO6" s="135"/>
+      <c r="AP6" s="134"/>
+      <c r="AQ6" s="135"/>
+      <c r="AR6" s="135"/>
+      <c r="AS6" s="135"/>
+      <c r="AT6" s="134"/>
+      <c r="AU6" s="135"/>
+      <c r="AV6" s="135"/>
+      <c r="AW6" s="135"/>
+      <c r="AX6" s="134"/>
+      <c r="AY6" s="135"/>
+      <c r="AZ6" s="135"/>
+      <c r="BA6" s="135"/>
       <c r="BE6" s="86"/>
     </row>
     <row r="7" spans="2:57" s="27" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3061,7 +3061,7 @@
     </row>
     <row r="9" spans="2:57" s="18" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="19"/>
-      <c r="C9" s="146" t="s">
+      <c r="C9" s="120" t="s">
         <v>30</v>
       </c>
       <c r="D9" s="41">
@@ -3128,7 +3128,7 @@
     </row>
     <row r="10" spans="2:57" s="18" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="19"/>
-      <c r="C10" s="146"/>
+      <c r="C10" s="120"/>
       <c r="D10" s="43"/>
       <c r="E10" s="44">
         <f>SUM(F10:BA10)</f>
@@ -3193,7 +3193,7 @@
     </row>
     <row r="11" spans="2:57" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="19"/>
-      <c r="C11" s="146" t="s">
+      <c r="C11" s="120" t="s">
         <v>31</v>
       </c>
       <c r="D11" s="41">
@@ -3260,7 +3260,7 @@
     </row>
     <row r="12" spans="2:57" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="19"/>
-      <c r="C12" s="146"/>
+      <c r="C12" s="120"/>
       <c r="D12" s="43"/>
       <c r="E12" s="44">
         <f>SUM(F12:BA12)</f>
@@ -3325,7 +3325,7 @@
     </row>
     <row r="13" spans="2:57" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="19"/>
-      <c r="C13" s="146" t="s">
+      <c r="C13" s="120" t="s">
         <v>32</v>
       </c>
       <c r="D13" s="41">
@@ -3392,7 +3392,7 @@
     </row>
     <row r="14" spans="2:57" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="19"/>
-      <c r="C14" s="146"/>
+      <c r="C14" s="120"/>
       <c r="D14" s="43"/>
       <c r="E14" s="44">
         <f>SUM(F14:BA14)</f>
@@ -3457,7 +3457,7 @@
     </row>
     <row r="15" spans="2:57" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="19"/>
-      <c r="C15" s="146" t="s">
+      <c r="C15" s="120" t="s">
         <v>33</v>
       </c>
       <c r="D15" s="41">
@@ -3524,7 +3524,7 @@
     </row>
     <row r="16" spans="2:57" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="19"/>
-      <c r="C16" s="146"/>
+      <c r="C16" s="120"/>
       <c r="D16" s="43"/>
       <c r="E16" s="44">
         <f>SUM(F16:BA16)</f>
@@ -3589,7 +3589,7 @@
     </row>
     <row r="17" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="19"/>
-      <c r="C17" s="146" t="s">
+      <c r="C17" s="120" t="s">
         <v>34</v>
       </c>
       <c r="D17" s="41">
@@ -3656,7 +3656,7 @@
     </row>
     <row r="18" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="19"/>
-      <c r="C18" s="146"/>
+      <c r="C18" s="120"/>
       <c r="D18" s="43"/>
       <c r="E18" s="44">
         <f>SUM(F18:BA18)</f>
@@ -3721,7 +3721,7 @@
     </row>
     <row r="19" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="19"/>
-      <c r="C19" s="146"/>
+      <c r="C19" s="120"/>
       <c r="D19" s="41"/>
       <c r="E19" s="42"/>
       <c r="F19" s="7"/>
@@ -3775,7 +3775,7 @@
     </row>
     <row r="20" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="19"/>
-      <c r="C20" s="146"/>
+      <c r="C20" s="120"/>
       <c r="D20" s="43"/>
       <c r="E20" s="44"/>
       <c r="F20" s="7"/>
@@ -3939,7 +3939,7 @@
     </row>
     <row r="23" spans="2:53" s="18" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B23" s="19"/>
-      <c r="C23" s="147" t="s">
+      <c r="C23" s="131" t="s">
         <v>25</v>
       </c>
       <c r="D23" s="41">
@@ -4006,7 +4006,7 @@
     </row>
     <row r="24" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="19"/>
-      <c r="C24" s="148"/>
+      <c r="C24" s="132"/>
       <c r="D24" s="43"/>
       <c r="E24" s="44">
         <f>SUM(F24:BA24)</f>
@@ -4071,7 +4071,7 @@
     </row>
     <row r="25" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="19"/>
-      <c r="C25" s="146" t="s">
+      <c r="C25" s="120" t="s">
         <v>24</v>
       </c>
       <c r="D25" s="41">
@@ -4138,7 +4138,7 @@
     </row>
     <row r="26" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="19"/>
-      <c r="C26" s="146"/>
+      <c r="C26" s="120"/>
       <c r="D26" s="43"/>
       <c r="E26" s="44">
         <f>SUM(F26:BA26)</f>
@@ -4203,7 +4203,7 @@
     </row>
     <row r="27" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="19"/>
-      <c r="C27" s="146" t="s">
+      <c r="C27" s="120" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="41">
@@ -4270,7 +4270,7 @@
     </row>
     <row r="28" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="19"/>
-      <c r="C28" s="146"/>
+      <c r="C28" s="120"/>
       <c r="D28" s="43"/>
       <c r="E28" s="44">
         <f>SUM(F28:BA28)</f>
@@ -4335,7 +4335,7 @@
     </row>
     <row r="29" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="19"/>
-      <c r="C29" s="146" t="s">
+      <c r="C29" s="120" t="s">
         <v>26</v>
       </c>
       <c r="D29" s="41">
@@ -4402,7 +4402,7 @@
     </row>
     <row r="30" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="19"/>
-      <c r="C30" s="146"/>
+      <c r="C30" s="120"/>
       <c r="D30" s="43"/>
       <c r="E30" s="44">
         <f>SUM(F30:BA30)</f>
@@ -4469,7 +4469,7 @@
     </row>
     <row r="31" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="19"/>
-      <c r="C31" s="146" t="s">
+      <c r="C31" s="120" t="s">
         <v>27</v>
       </c>
       <c r="D31" s="41">
@@ -4536,7 +4536,7 @@
     </row>
     <row r="32" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="19"/>
-      <c r="C32" s="146"/>
+      <c r="C32" s="120"/>
       <c r="D32" s="43"/>
       <c r="E32" s="44">
         <f>SUM(F32:BA32)</f>
@@ -4601,7 +4601,7 @@
     </row>
     <row r="33" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="19"/>
-      <c r="C33" s="146" t="s">
+      <c r="C33" s="120" t="s">
         <v>28</v>
       </c>
       <c r="D33" s="41">
@@ -4668,7 +4668,7 @@
     </row>
     <row r="34" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="19"/>
-      <c r="C34" s="146"/>
+      <c r="C34" s="120"/>
       <c r="D34" s="43"/>
       <c r="E34" s="44">
         <f>SUM(F34:BA34)</f>
@@ -4733,7 +4733,7 @@
     </row>
     <row r="35" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="19"/>
-      <c r="C35" s="149" t="s">
+      <c r="C35" s="121" t="s">
         <v>29</v>
       </c>
       <c r="D35" s="41">
@@ -4800,7 +4800,7 @@
     </row>
     <row r="36" spans="2:53" s="18" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="19"/>
-      <c r="C36" s="149"/>
+      <c r="C36" s="121"/>
       <c r="D36" s="43"/>
       <c r="E36" s="44">
         <f>SUM(F36:BA36)</f>
@@ -4975,7 +4975,7 @@
     </row>
     <row r="39" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="19"/>
-      <c r="C39" s="146" t="s">
+      <c r="C39" s="120" t="s">
         <v>35</v>
       </c>
       <c r="D39" s="41">
@@ -5050,11 +5050,11 @@
     </row>
     <row r="40" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="19"/>
-      <c r="C40" s="146"/>
+      <c r="C40" s="120"/>
       <c r="D40" s="43"/>
       <c r="E40" s="44">
         <f>SUM(F40:BA40)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F40" s="7"/>
       <c r="G40" s="5"/>
@@ -5076,10 +5076,18 @@
       <c r="Q40" s="108">
         <v>0</v>
       </c>
-      <c r="R40" s="106"/>
-      <c r="S40" s="107"/>
-      <c r="T40" s="107"/>
-      <c r="U40" s="108"/>
+      <c r="R40" s="106">
+        <v>0.5</v>
+      </c>
+      <c r="S40" s="107">
+        <v>1.5</v>
+      </c>
+      <c r="T40" s="107">
+        <v>0</v>
+      </c>
+      <c r="U40" s="108">
+        <v>0</v>
+      </c>
       <c r="V40" s="7"/>
       <c r="W40" s="5"/>
       <c r="X40" s="5"/>
@@ -5115,7 +5123,7 @@
     </row>
     <row r="41" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="19"/>
-      <c r="C41" s="146" t="s">
+      <c r="C41" s="120" t="s">
         <v>36</v>
       </c>
       <c r="D41" s="41">
@@ -5190,11 +5198,11 @@
     </row>
     <row r="42" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="19"/>
-      <c r="C42" s="146"/>
+      <c r="C42" s="120"/>
       <c r="D42" s="43"/>
       <c r="E42" s="44">
         <f>SUM(F42:BA42)</f>
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="F42" s="7"/>
       <c r="G42" s="5"/>
@@ -5216,10 +5224,18 @@
       <c r="Q42" s="108">
         <v>0</v>
       </c>
-      <c r="R42" s="106"/>
-      <c r="S42" s="107"/>
-      <c r="T42" s="107"/>
-      <c r="U42" s="108"/>
+      <c r="R42" s="106">
+        <v>1</v>
+      </c>
+      <c r="S42" s="107">
+        <v>0.25</v>
+      </c>
+      <c r="T42" s="107">
+        <v>0</v>
+      </c>
+      <c r="U42" s="108">
+        <v>0</v>
+      </c>
       <c r="V42" s="7"/>
       <c r="W42" s="5"/>
       <c r="X42" s="5"/>
@@ -5255,7 +5271,7 @@
     </row>
     <row r="43" spans="2:53" s="18" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B43" s="19"/>
-      <c r="C43" s="147" t="s">
+      <c r="C43" s="131" t="s">
         <v>37</v>
       </c>
       <c r="D43" s="41">
@@ -5330,11 +5346,11 @@
     </row>
     <row r="44" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="19"/>
-      <c r="C44" s="148"/>
+      <c r="C44" s="132"/>
       <c r="D44" s="43"/>
       <c r="E44" s="44">
         <f>SUM(F44:BA44)</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F44" s="7"/>
       <c r="G44" s="5"/>
@@ -5356,10 +5372,18 @@
       <c r="Q44" s="108">
         <v>0</v>
       </c>
-      <c r="R44" s="106"/>
-      <c r="S44" s="107"/>
-      <c r="T44" s="107"/>
-      <c r="U44" s="108"/>
+      <c r="R44" s="106">
+        <v>0.2</v>
+      </c>
+      <c r="S44" s="107">
+        <v>0</v>
+      </c>
+      <c r="T44" s="107">
+        <v>0</v>
+      </c>
+      <c r="U44" s="108">
+        <v>0</v>
+      </c>
       <c r="V44" s="7"/>
       <c r="W44" s="5"/>
       <c r="X44" s="5"/>
@@ -5395,7 +5419,7 @@
     </row>
     <row r="45" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B45" s="19"/>
-      <c r="C45" s="146" t="s">
+      <c r="C45" s="120" t="s">
         <v>38</v>
       </c>
       <c r="D45" s="41">
@@ -5470,11 +5494,11 @@
     </row>
     <row r="46" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="19"/>
-      <c r="C46" s="146"/>
+      <c r="C46" s="120"/>
       <c r="D46" s="43"/>
       <c r="E46" s="44">
         <f>SUM(F46:BA46)</f>
-        <v>1.55</v>
+        <v>3.1</v>
       </c>
       <c r="F46" s="7"/>
       <c r="G46" s="5"/>
@@ -5496,10 +5520,18 @@
       <c r="Q46" s="108">
         <v>1</v>
       </c>
-      <c r="R46" s="106"/>
-      <c r="S46" s="107"/>
-      <c r="T46" s="107"/>
-      <c r="U46" s="108"/>
+      <c r="R46" s="106">
+        <v>0</v>
+      </c>
+      <c r="S46" s="107">
+        <v>0.25</v>
+      </c>
+      <c r="T46" s="107">
+        <v>0</v>
+      </c>
+      <c r="U46" s="108">
+        <v>1.3</v>
+      </c>
       <c r="V46" s="7"/>
       <c r="W46" s="5"/>
       <c r="X46" s="5"/>
@@ -5535,7 +5567,7 @@
     </row>
     <row r="47" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="19"/>
-      <c r="C47" s="146" t="s">
+      <c r="C47" s="120" t="s">
         <v>39</v>
       </c>
       <c r="D47" s="41">
@@ -5610,11 +5642,11 @@
     </row>
     <row r="48" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B48" s="19"/>
-      <c r="C48" s="146"/>
+      <c r="C48" s="120"/>
       <c r="D48" s="43"/>
       <c r="E48" s="44">
         <f>SUM(F48:BA48)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F48" s="7"/>
       <c r="G48" s="5"/>
@@ -5636,10 +5668,18 @@
       <c r="Q48" s="108">
         <v>0</v>
       </c>
-      <c r="R48" s="106"/>
-      <c r="S48" s="107"/>
-      <c r="T48" s="107"/>
-      <c r="U48" s="108"/>
+      <c r="R48" s="106">
+        <v>1</v>
+      </c>
+      <c r="S48" s="107">
+        <v>1</v>
+      </c>
+      <c r="T48" s="107">
+        <v>1</v>
+      </c>
+      <c r="U48" s="108">
+        <v>0</v>
+      </c>
       <c r="V48" s="7"/>
       <c r="W48" s="5"/>
       <c r="X48" s="5"/>
@@ -5675,7 +5715,7 @@
     </row>
     <row r="49" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B49" s="19"/>
-      <c r="C49" s="146" t="s">
+      <c r="C49" s="120" t="s">
         <v>40</v>
       </c>
       <c r="D49" s="41">
@@ -5750,11 +5790,11 @@
     </row>
     <row r="50" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B50" s="19"/>
-      <c r="C50" s="146"/>
+      <c r="C50" s="120"/>
       <c r="D50" s="43"/>
       <c r="E50" s="44">
         <f>SUM(F50:BA50)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F50" s="7"/>
       <c r="G50" s="5"/>
@@ -5776,10 +5816,18 @@
       <c r="Q50" s="108">
         <v>1</v>
       </c>
-      <c r="R50" s="106"/>
-      <c r="S50" s="107"/>
-      <c r="T50" s="107"/>
-      <c r="U50" s="108"/>
+      <c r="R50" s="106">
+        <v>1</v>
+      </c>
+      <c r="S50" s="107">
+        <v>1</v>
+      </c>
+      <c r="T50" s="107">
+        <v>1</v>
+      </c>
+      <c r="U50" s="108">
+        <v>1</v>
+      </c>
       <c r="V50" s="7"/>
       <c r="W50" s="5"/>
       <c r="X50" s="5"/>
@@ -5815,7 +5863,7 @@
     </row>
     <row r="51" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="19"/>
-      <c r="C51" s="149" t="s">
+      <c r="C51" s="121" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="41">
@@ -5890,11 +5938,11 @@
     </row>
     <row r="52" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B52" s="19"/>
-      <c r="C52" s="149"/>
+      <c r="C52" s="121"/>
       <c r="D52" s="43"/>
       <c r="E52" s="44">
         <f>SUM(F52:BA52)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F52" s="7"/>
       <c r="G52" s="5"/>
@@ -5916,10 +5964,18 @@
       <c r="Q52" s="108">
         <v>0.5</v>
       </c>
-      <c r="R52" s="106"/>
-      <c r="S52" s="107"/>
-      <c r="T52" s="107"/>
-      <c r="U52" s="108"/>
+      <c r="R52" s="106">
+        <v>0.5</v>
+      </c>
+      <c r="S52" s="107">
+        <v>0.5</v>
+      </c>
+      <c r="T52" s="107">
+        <v>0.5</v>
+      </c>
+      <c r="U52" s="108">
+        <v>0.5</v>
+      </c>
       <c r="V52" s="7"/>
       <c r="W52" s="5"/>
       <c r="X52" s="5"/>
@@ -5955,7 +6011,7 @@
     </row>
     <row r="53" spans="2:53" s="18" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B53" s="19"/>
-      <c r="C53" s="149"/>
+      <c r="C53" s="121"/>
       <c r="D53" s="41">
         <f>SUM(F53:BA53)</f>
         <v>0</v>
@@ -6012,7 +6068,7 @@
     </row>
     <row r="54" spans="2:53" s="18" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B54" s="19"/>
-      <c r="C54" s="149"/>
+      <c r="C54" s="121"/>
       <c r="D54" s="43"/>
       <c r="E54" s="44">
         <f>SUM(F54:BA54)</f>
@@ -6179,7 +6235,7 @@
     </row>
     <row r="57" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="19"/>
-      <c r="C57" s="146" t="s">
+      <c r="C57" s="120" t="s">
         <v>41</v>
       </c>
       <c r="D57" s="41">
@@ -6254,11 +6310,11 @@
     </row>
     <row r="58" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B58" s="19"/>
-      <c r="C58" s="146"/>
+      <c r="C58" s="120"/>
       <c r="D58" s="43"/>
       <c r="E58" s="44">
         <f>SUM(F58:BA58)</f>
-        <v>0</v>
+        <v>4.45</v>
       </c>
       <c r="F58" s="7"/>
       <c r="G58" s="5"/>
@@ -6276,10 +6332,18 @@
       <c r="S58" s="5"/>
       <c r="T58" s="5"/>
       <c r="U58" s="6"/>
-      <c r="V58" s="115"/>
-      <c r="W58" s="116"/>
-      <c r="X58" s="116"/>
-      <c r="Y58" s="117"/>
+      <c r="V58" s="115">
+        <v>1</v>
+      </c>
+      <c r="W58" s="116">
+        <v>1.45</v>
+      </c>
+      <c r="X58" s="116">
+        <v>0</v>
+      </c>
+      <c r="Y58" s="117">
+        <v>2</v>
+      </c>
       <c r="Z58" s="115"/>
       <c r="AA58" s="116"/>
       <c r="AB58" s="116"/>
@@ -6311,7 +6375,7 @@
     </row>
     <row r="59" spans="2:53" s="18" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B59" s="19"/>
-      <c r="C59" s="146" t="s">
+      <c r="C59" s="120" t="s">
         <v>42</v>
       </c>
       <c r="D59" s="41">
@@ -6386,11 +6450,11 @@
     </row>
     <row r="60" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B60" s="19"/>
-      <c r="C60" s="146"/>
+      <c r="C60" s="120"/>
       <c r="D60" s="43"/>
       <c r="E60" s="44">
         <f>SUM(F60:BA60)</f>
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="F60" s="7"/>
       <c r="G60" s="5"/>
@@ -6408,10 +6472,18 @@
       <c r="S60" s="5"/>
       <c r="T60" s="5"/>
       <c r="U60" s="6"/>
-      <c r="V60" s="115"/>
-      <c r="W60" s="116"/>
-      <c r="X60" s="116"/>
-      <c r="Y60" s="117"/>
+      <c r="V60" s="115">
+        <v>1</v>
+      </c>
+      <c r="W60" s="116">
+        <v>1</v>
+      </c>
+      <c r="X60" s="116">
+        <v>0</v>
+      </c>
+      <c r="Y60" s="117">
+        <v>0.25</v>
+      </c>
       <c r="Z60" s="115"/>
       <c r="AA60" s="116"/>
       <c r="AB60" s="116"/>
@@ -6443,7 +6515,7 @@
     </row>
     <row r="61" spans="2:53" s="18" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B61" s="19"/>
-      <c r="C61" s="146" t="s">
+      <c r="C61" s="120" t="s">
         <v>43</v>
       </c>
       <c r="D61" s="41">
@@ -6518,11 +6590,11 @@
     </row>
     <row r="62" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B62" s="19"/>
-      <c r="C62" s="146"/>
+      <c r="C62" s="120"/>
       <c r="D62" s="43"/>
       <c r="E62" s="44">
         <f>SUM(F62:BA62)</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="F62" s="7"/>
       <c r="G62" s="5"/>
@@ -6540,10 +6612,18 @@
       <c r="S62" s="5"/>
       <c r="T62" s="5"/>
       <c r="U62" s="6"/>
-      <c r="V62" s="115"/>
-      <c r="W62" s="116"/>
-      <c r="X62" s="116"/>
-      <c r="Y62" s="117"/>
+      <c r="V62" s="115">
+        <v>1</v>
+      </c>
+      <c r="W62" s="116">
+        <v>1</v>
+      </c>
+      <c r="X62" s="116">
+        <v>1</v>
+      </c>
+      <c r="Y62" s="117">
+        <v>0.5</v>
+      </c>
       <c r="Z62" s="115"/>
       <c r="AA62" s="116"/>
       <c r="AB62" s="116"/>
@@ -6575,7 +6655,7 @@
     </row>
     <row r="63" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B63" s="19"/>
-      <c r="C63" s="146" t="s">
+      <c r="C63" s="120" t="s">
         <v>44</v>
       </c>
       <c r="D63" s="41">
@@ -6650,11 +6730,11 @@
     </row>
     <row r="64" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B64" s="19"/>
-      <c r="C64" s="146"/>
+      <c r="C64" s="120"/>
       <c r="D64" s="43"/>
       <c r="E64" s="44">
         <f>SUM(F64:BA64)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F64" s="7"/>
       <c r="G64" s="5"/>
@@ -6672,10 +6752,18 @@
       <c r="S64" s="5"/>
       <c r="T64" s="5"/>
       <c r="U64" s="6"/>
-      <c r="V64" s="115"/>
-      <c r="W64" s="116"/>
-      <c r="X64" s="116"/>
-      <c r="Y64" s="117"/>
+      <c r="V64" s="115">
+        <v>0</v>
+      </c>
+      <c r="W64" s="116">
+        <v>1</v>
+      </c>
+      <c r="X64" s="116">
+        <v>1</v>
+      </c>
+      <c r="Y64" s="117">
+        <v>1</v>
+      </c>
       <c r="Z64" s="115"/>
       <c r="AA64" s="116"/>
       <c r="AB64" s="116"/>
@@ -6707,7 +6795,7 @@
     </row>
     <row r="65" spans="2:53" s="18" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B65" s="19"/>
-      <c r="C65" s="146" t="s">
+      <c r="C65" s="120" t="s">
         <v>45</v>
       </c>
       <c r="D65" s="41">
@@ -6782,7 +6870,7 @@
     </row>
     <row r="66" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B66" s="19"/>
-      <c r="C66" s="146"/>
+      <c r="C66" s="120"/>
       <c r="D66" s="43"/>
       <c r="E66" s="44">
         <f>SUM(F66:BA66)</f>
@@ -6804,10 +6892,18 @@
       <c r="S66" s="5"/>
       <c r="T66" s="5"/>
       <c r="U66" s="6"/>
-      <c r="V66" s="115"/>
-      <c r="W66" s="116"/>
-      <c r="X66" s="116"/>
-      <c r="Y66" s="117"/>
+      <c r="V66" s="115">
+        <v>0</v>
+      </c>
+      <c r="W66" s="116">
+        <v>0</v>
+      </c>
+      <c r="X66" s="116">
+        <v>0</v>
+      </c>
+      <c r="Y66" s="117">
+        <v>0</v>
+      </c>
       <c r="Z66" s="115"/>
       <c r="AA66" s="116"/>
       <c r="AB66" s="116"/>
@@ -6839,7 +6935,7 @@
     </row>
     <row r="67" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B67" s="19"/>
-      <c r="C67" s="146" t="s">
+      <c r="C67" s="120" t="s">
         <v>29</v>
       </c>
       <c r="D67" s="41">
@@ -6914,11 +7010,11 @@
     </row>
     <row r="68" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B68" s="19"/>
-      <c r="C68" s="146"/>
+      <c r="C68" s="120"/>
       <c r="D68" s="43"/>
       <c r="E68" s="44">
         <f>SUM(F68:BA68)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="F68" s="7"/>
       <c r="G68" s="5"/>
@@ -6936,10 +7032,18 @@
       <c r="S68" s="5"/>
       <c r="T68" s="5"/>
       <c r="U68" s="6"/>
-      <c r="V68" s="115"/>
-      <c r="W68" s="116"/>
-      <c r="X68" s="116"/>
-      <c r="Y68" s="117"/>
+      <c r="V68" s="115">
+        <v>0.2</v>
+      </c>
+      <c r="W68" s="116">
+        <v>0.2</v>
+      </c>
+      <c r="X68" s="116">
+        <v>0.2</v>
+      </c>
+      <c r="Y68" s="117">
+        <v>0.2</v>
+      </c>
       <c r="Z68" s="115"/>
       <c r="AA68" s="116"/>
       <c r="AB68" s="116"/>
@@ -6971,7 +7075,7 @@
     </row>
     <row r="69" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B69" s="19"/>
-      <c r="C69" s="149"/>
+      <c r="C69" s="121"/>
       <c r="D69" s="41">
         <f>SUM(F69:BA69)</f>
         <v>0</v>
@@ -7028,7 +7132,7 @@
     </row>
     <row r="70" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B70" s="19"/>
-      <c r="C70" s="149"/>
+      <c r="C70" s="121"/>
       <c r="D70" s="43"/>
       <c r="E70" s="44">
         <f>SUM(F70:BA70)</f>
@@ -7085,7 +7189,7 @@
     </row>
     <row r="71" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B71" s="19"/>
-      <c r="C71" s="149"/>
+      <c r="C71" s="121"/>
       <c r="D71" s="41">
         <f>SUM(F71:BA71)</f>
         <v>0</v>
@@ -7142,7 +7246,7 @@
     </row>
     <row r="72" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B72" s="19"/>
-      <c r="C72" s="149"/>
+      <c r="C72" s="121"/>
       <c r="D72" s="43"/>
       <c r="E72" s="44">
         <f>SUM(F72:BA72)</f>
@@ -7307,7 +7411,7 @@
     </row>
     <row r="75" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B75" s="19"/>
-      <c r="C75" s="146"/>
+      <c r="C75" s="120"/>
       <c r="D75" s="41">
         <f>SUM(F75:BA75)</f>
         <v>0</v>
@@ -7364,7 +7468,7 @@
     </row>
     <row r="76" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B76" s="19"/>
-      <c r="C76" s="146"/>
+      <c r="C76" s="120"/>
       <c r="D76" s="43"/>
       <c r="E76" s="44">
         <f>SUM(F76:BA76)</f>
@@ -7421,7 +7525,7 @@
     </row>
     <row r="77" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B77" s="19"/>
-      <c r="C77" s="146"/>
+      <c r="C77" s="120"/>
       <c r="D77" s="41">
         <f>SUM(F77:BA77)</f>
         <v>0</v>
@@ -7478,7 +7582,7 @@
     </row>
     <row r="78" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B78" s="19"/>
-      <c r="C78" s="146"/>
+      <c r="C78" s="120"/>
       <c r="D78" s="43"/>
       <c r="E78" s="44">
         <f>SUM(F78:BA78)</f>
@@ -7535,7 +7639,7 @@
     </row>
     <row r="79" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B79" s="19"/>
-      <c r="C79" s="146"/>
+      <c r="C79" s="120"/>
       <c r="D79" s="41">
         <f>SUM(F79:BA79)</f>
         <v>0</v>
@@ -7592,7 +7696,7 @@
     </row>
     <row r="80" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B80" s="19"/>
-      <c r="C80" s="146"/>
+      <c r="C80" s="120"/>
       <c r="D80" s="43"/>
       <c r="E80" s="44">
         <f>SUM(F80:BA80)</f>
@@ -7649,7 +7753,7 @@
     </row>
     <row r="81" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B81" s="19"/>
-      <c r="C81" s="146"/>
+      <c r="C81" s="120"/>
       <c r="D81" s="41">
         <f>SUM(F81:BA81)</f>
         <v>0</v>
@@ -7706,7 +7810,7 @@
     </row>
     <row r="82" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B82" s="19"/>
-      <c r="C82" s="146"/>
+      <c r="C82" s="120"/>
       <c r="D82" s="43"/>
       <c r="E82" s="44">
         <f>SUM(F82:BA82)</f>
@@ -7871,7 +7975,7 @@
     </row>
     <row r="85" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B85" s="19"/>
-      <c r="C85" s="146"/>
+      <c r="C85" s="120"/>
       <c r="D85" s="41">
         <f>SUM(F85:BA85)</f>
         <v>0</v>
@@ -7928,7 +8032,7 @@
     </row>
     <row r="86" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B86" s="19"/>
-      <c r="C86" s="146"/>
+      <c r="C86" s="120"/>
       <c r="D86" s="43"/>
       <c r="E86" s="44">
         <f>SUM(F86:BA86)</f>
@@ -7985,7 +8089,7 @@
     </row>
     <row r="87" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B87" s="19"/>
-      <c r="C87" s="146"/>
+      <c r="C87" s="120"/>
       <c r="D87" s="41">
         <f>SUM(F87:BA87)</f>
         <v>0</v>
@@ -8042,7 +8146,7 @@
     </row>
     <row r="88" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B88" s="19"/>
-      <c r="C88" s="146"/>
+      <c r="C88" s="120"/>
       <c r="D88" s="43"/>
       <c r="E88" s="44">
         <f>SUM(F88:BA88)</f>
@@ -8099,7 +8203,7 @@
     </row>
     <row r="89" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B89" s="19"/>
-      <c r="C89" s="146"/>
+      <c r="C89" s="120"/>
       <c r="D89" s="41">
         <f>SUM(F89:BA89)</f>
         <v>0</v>
@@ -8156,7 +8260,7 @@
     </row>
     <row r="90" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B90" s="19"/>
-      <c r="C90" s="146"/>
+      <c r="C90" s="120"/>
       <c r="D90" s="43"/>
       <c r="E90" s="44">
         <f>SUM(F90:BA90)</f>
@@ -8213,7 +8317,7 @@
     </row>
     <row r="91" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B91" s="19"/>
-      <c r="C91" s="146"/>
+      <c r="C91" s="120"/>
       <c r="D91" s="41">
         <f>SUM(F91:BA91)</f>
         <v>0</v>
@@ -8270,7 +8374,7 @@
     </row>
     <row r="92" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B92" s="19"/>
-      <c r="C92" s="146"/>
+      <c r="C92" s="120"/>
       <c r="D92" s="43"/>
       <c r="E92" s="44">
         <f>SUM(F92:BA92)</f>
@@ -8435,7 +8539,7 @@
     </row>
     <row r="95" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B95" s="19"/>
-      <c r="C95" s="146"/>
+      <c r="C95" s="120"/>
       <c r="D95" s="41">
         <f>SUM(F95:BA95)</f>
         <v>0</v>
@@ -8492,7 +8596,7 @@
     </row>
     <row r="96" spans="2:53" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B96" s="19"/>
-      <c r="C96" s="146"/>
+      <c r="C96" s="120"/>
       <c r="D96" s="43"/>
       <c r="E96" s="44">
         <f>SUM(F96:BA96)</f>
@@ -8549,7 +8653,7 @@
     </row>
     <row r="97" spans="2:74" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B97" s="19"/>
-      <c r="C97" s="146"/>
+      <c r="C97" s="120"/>
       <c r="D97" s="41">
         <f>SUM(F97:BA97)</f>
         <v>0</v>
@@ -8606,7 +8710,7 @@
     </row>
     <row r="98" spans="2:74" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B98" s="19"/>
-      <c r="C98" s="146"/>
+      <c r="C98" s="120"/>
       <c r="D98" s="43"/>
       <c r="E98" s="44">
         <f>SUM(F98:BA98)</f>
@@ -8771,7 +8875,7 @@
     </row>
     <row r="101" spans="2:74" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B101" s="19"/>
-      <c r="C101" s="150"/>
+      <c r="C101" s="124"/>
       <c r="D101" s="41">
         <f>SUM(F101:BA101)</f>
         <v>0</v>
@@ -8828,7 +8932,7 @@
     </row>
     <row r="102" spans="2:74" s="18" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B102" s="19"/>
-      <c r="C102" s="150"/>
+      <c r="C102" s="124"/>
       <c r="D102" s="43"/>
       <c r="E102" s="44">
         <f>SUM(F102:BA102)</f>
@@ -8990,11 +9094,11 @@
       <c r="AY104" s="5"/>
       <c r="AZ104" s="5"/>
       <c r="BA104" s="6"/>
-      <c r="BE104" s="119" t="s">
+      <c r="BE104" s="141" t="s">
         <v>10</v>
       </c>
-      <c r="BF104" s="120"/>
-      <c r="BG104" s="121"/>
+      <c r="BF104" s="142"/>
+      <c r="BG104" s="143"/>
       <c r="BH104" s="55">
         <f>SUM(D9:D105)</f>
         <v>84</v>
@@ -9007,7 +9111,7 @@
     </row>
     <row r="105" spans="2:74" s="18" customFormat="1" ht="19.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B105" s="19"/>
-      <c r="C105" s="150"/>
+      <c r="C105" s="124"/>
       <c r="D105" s="41">
         <f>SUM(F105:BA105)</f>
         <v>0</v>
@@ -9061,15 +9165,15 @@
       <c r="AY105" s="5"/>
       <c r="AZ105" s="5"/>
       <c r="BA105" s="5"/>
-      <c r="BE105" s="119" t="s">
+      <c r="BE105" s="141" t="s">
         <v>9</v>
       </c>
-      <c r="BF105" s="120"/>
-      <c r="BG105" s="121"/>
+      <c r="BF105" s="142"/>
+      <c r="BG105" s="143"/>
       <c r="BH105" s="58"/>
       <c r="BI105" s="55">
         <f>SUM(E9:E106)</f>
-        <v>42.75</v>
+        <v>70.75</v>
       </c>
       <c r="BJ105" s="57" t="s">
         <v>11</v>
@@ -9078,7 +9182,7 @@
     </row>
     <row r="106" spans="2:74" s="18" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B106" s="19"/>
-      <c r="C106" s="150"/>
+      <c r="C106" s="124"/>
       <c r="D106" s="43"/>
       <c r="E106" s="44">
         <f>SUM(F106:BA106)</f>
@@ -9151,20 +9255,20 @@
       </c>
       <c r="E107" s="61">
         <f>SUM(E9:E106)</f>
-        <v>42.75</v>
+        <v>70.75</v>
       </c>
       <c r="BB107" s="29"/>
       <c r="BC107" s="29"/>
-      <c r="BE107" s="119" t="s">
+      <c r="BE107" s="141" t="s">
         <v>1</v>
       </c>
-      <c r="BF107" s="120"/>
-      <c r="BG107" s="121"/>
-      <c r="BH107" s="151">
+      <c r="BF107" s="142"/>
+      <c r="BG107" s="143"/>
+      <c r="BH107" s="125">
         <f>IF((BH104-BI105)&gt;0,(BH104-BI105),(BH104-BI105)*(1))</f>
-        <v>41.25</v>
-      </c>
-      <c r="BI107" s="152"/>
+        <v>13.25</v>
+      </c>
+      <c r="BI107" s="126"/>
       <c r="BJ107" s="57" t="s">
         <v>11</v>
       </c>
@@ -9174,38 +9278,38 @@
       <c r="B108" s="28"/>
       <c r="D108" s="80"/>
       <c r="E108" s="81"/>
-      <c r="F108" s="124" t="s">
+      <c r="F108" s="146" t="s">
         <v>4</v>
       </c>
-      <c r="G108" s="124"/>
-      <c r="H108" s="124"/>
-      <c r="I108" s="125"/>
-      <c r="J108" s="126" t="s">
+      <c r="G108" s="146"/>
+      <c r="H108" s="146"/>
+      <c r="I108" s="147"/>
+      <c r="J108" s="148" t="s">
         <v>5</v>
       </c>
-      <c r="K108" s="127"/>
-      <c r="L108" s="127"/>
-      <c r="M108" s="127"/>
-      <c r="N108" s="128" t="s">
+      <c r="K108" s="149"/>
+      <c r="L108" s="149"/>
+      <c r="M108" s="149"/>
+      <c r="N108" s="150" t="s">
         <v>6</v>
       </c>
-      <c r="O108" s="128"/>
-      <c r="P108" s="128"/>
-      <c r="Q108" s="128"/>
-      <c r="R108" s="128"/>
-      <c r="S108" s="128"/>
-      <c r="T108" s="128"/>
-      <c r="U108" s="128"/>
-      <c r="V108" s="129" t="s">
+      <c r="O108" s="150"/>
+      <c r="P108" s="150"/>
+      <c r="Q108" s="150"/>
+      <c r="R108" s="150"/>
+      <c r="S108" s="150"/>
+      <c r="T108" s="150"/>
+      <c r="U108" s="150"/>
+      <c r="V108" s="151" t="s">
         <v>2</v>
       </c>
-      <c r="W108" s="129"/>
-      <c r="X108" s="129"/>
-      <c r="Y108" s="129"/>
-      <c r="Z108" s="129"/>
-      <c r="AA108" s="129"/>
-      <c r="AB108" s="129"/>
-      <c r="AC108" s="129"/>
+      <c r="W108" s="151"/>
+      <c r="X108" s="151"/>
+      <c r="Y108" s="151"/>
+      <c r="Z108" s="151"/>
+      <c r="AA108" s="151"/>
+      <c r="AB108" s="151"/>
+      <c r="AC108" s="151"/>
       <c r="AL108" s="62"/>
       <c r="AM108" s="62"/>
       <c r="AN108" s="62"/>
@@ -9353,12 +9457,12 @@
       <c r="BB110" s="69"/>
       <c r="BC110" s="67"/>
       <c r="BD110" s="67"/>
-      <c r="BF110" s="145">
+      <c r="BF110" s="129">
         <f>IF((BH107)&lt;=0,(BH107/24)*(-1),BH107/24)</f>
-        <v>1.71875</v>
-      </c>
-      <c r="BG110" s="145"/>
-      <c r="BH110" s="145"/>
+        <v>0.55208333333333337</v>
+      </c>
+      <c r="BG110" s="129"/>
+      <c r="BH110" s="129"/>
       <c r="BI110" s="40"/>
     </row>
     <row r="111" spans="2:74" s="18" customFormat="1" ht="18" x14ac:dyDescent="0.2">
@@ -10061,24 +10165,78 @@
     </row>
   </sheetData>
   <mergeCells count="114">
-    <mergeCell ref="N5:Q5"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="C95:C96"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="AT2:AW2"/>
+    <mergeCell ref="BE107:BG107"/>
+    <mergeCell ref="BE105:BG105"/>
+    <mergeCell ref="BE104:BG104"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F108:I108"/>
+    <mergeCell ref="J108:M108"/>
+    <mergeCell ref="N108:U108"/>
+    <mergeCell ref="V108:AC108"/>
+    <mergeCell ref="AH5:AK5"/>
+    <mergeCell ref="AL5:AO5"/>
+    <mergeCell ref="AP5:AS5"/>
+    <mergeCell ref="Z5:AC5"/>
+    <mergeCell ref="AD5:AG5"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="N4:Q4"/>
+    <mergeCell ref="V4:Y4"/>
+    <mergeCell ref="V2:Y2"/>
+    <mergeCell ref="Z2:AC2"/>
+    <mergeCell ref="AD2:AG2"/>
+    <mergeCell ref="AH2:AK2"/>
+    <mergeCell ref="AL2:AO2"/>
+    <mergeCell ref="AL3:AO3"/>
+    <mergeCell ref="C1:BA1"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="N6:Q6"/>
+    <mergeCell ref="R6:U6"/>
+    <mergeCell ref="V6:Y6"/>
+    <mergeCell ref="Z6:AC6"/>
+    <mergeCell ref="AD6:AG6"/>
+    <mergeCell ref="AH6:AK6"/>
+    <mergeCell ref="AL6:AO6"/>
+    <mergeCell ref="AP6:AS6"/>
+    <mergeCell ref="AT6:AW6"/>
+    <mergeCell ref="AX6:BA6"/>
+    <mergeCell ref="AX2:BA2"/>
+    <mergeCell ref="AX3:BA3"/>
+    <mergeCell ref="AH3:AK3"/>
+    <mergeCell ref="AP2:AS2"/>
+    <mergeCell ref="AP3:AS3"/>
+    <mergeCell ref="R5:U5"/>
+    <mergeCell ref="V5:Y5"/>
+    <mergeCell ref="Z4:AC4"/>
+    <mergeCell ref="AD4:AG4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="BF110:BH110"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="J2:M2"/>
+    <mergeCell ref="N2:Q2"/>
+    <mergeCell ref="R2:U2"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="R4:U4"/>
+    <mergeCell ref="AT3:AW3"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="AH4:AK4"/>
+    <mergeCell ref="AL4:AO4"/>
+    <mergeCell ref="AP4:AS4"/>
     <mergeCell ref="Z3:AC3"/>
     <mergeCell ref="C105:C106"/>
     <mergeCell ref="C45:C46"/>
@@ -10103,78 +10261,24 @@
     <mergeCell ref="AD3:AG3"/>
     <mergeCell ref="C97:C98"/>
     <mergeCell ref="J5:M5"/>
-    <mergeCell ref="BF110:BH110"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="J2:M2"/>
-    <mergeCell ref="N2:Q2"/>
-    <mergeCell ref="R2:U2"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="R4:U4"/>
-    <mergeCell ref="AT3:AW3"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="AH4:AK4"/>
-    <mergeCell ref="AL4:AO4"/>
-    <mergeCell ref="AP4:AS4"/>
-    <mergeCell ref="C1:BA1"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="N6:Q6"/>
-    <mergeCell ref="R6:U6"/>
-    <mergeCell ref="V6:Y6"/>
-    <mergeCell ref="Z6:AC6"/>
-    <mergeCell ref="AD6:AG6"/>
-    <mergeCell ref="AH6:AK6"/>
-    <mergeCell ref="AL6:AO6"/>
-    <mergeCell ref="AP6:AS6"/>
-    <mergeCell ref="AT6:AW6"/>
-    <mergeCell ref="AX6:BA6"/>
-    <mergeCell ref="AX2:BA2"/>
-    <mergeCell ref="AX3:BA3"/>
-    <mergeCell ref="AH3:AK3"/>
-    <mergeCell ref="AP2:AS2"/>
-    <mergeCell ref="AP3:AS3"/>
-    <mergeCell ref="R5:U5"/>
-    <mergeCell ref="V5:Y5"/>
-    <mergeCell ref="Z4:AC4"/>
-    <mergeCell ref="AD4:AG4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="AT2:AW2"/>
-    <mergeCell ref="BE107:BG107"/>
-    <mergeCell ref="BE105:BG105"/>
-    <mergeCell ref="BE104:BG104"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="F108:I108"/>
-    <mergeCell ref="J108:M108"/>
-    <mergeCell ref="N108:U108"/>
-    <mergeCell ref="V108:AC108"/>
-    <mergeCell ref="AH5:AK5"/>
-    <mergeCell ref="AL5:AO5"/>
-    <mergeCell ref="AP5:AS5"/>
-    <mergeCell ref="Z5:AC5"/>
-    <mergeCell ref="AD5:AG5"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="V4:Y4"/>
-    <mergeCell ref="V2:Y2"/>
-    <mergeCell ref="Z2:AC2"/>
-    <mergeCell ref="AD2:AG2"/>
-    <mergeCell ref="AH2:AK2"/>
-    <mergeCell ref="AL2:AO2"/>
-    <mergeCell ref="AL3:AO3"/>
+    <mergeCell ref="N5:Q5"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="C95:C96"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="C85:C86"/>
   </mergeCells>
   <conditionalFormatting sqref="BF110">
     <cfRule type="expression" dxfId="1" priority="1">
@@ -10210,12 +10314,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="5030cb7a-6be5-477a-957d-975e4d3028a7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="83c7e37f-cb9c-4af6-99b9-72a827d5e6dc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10408,20 +10514,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="5030cb7a-6be5-477a-957d-975e4d3028a7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="83c7e37f-cb9c-4af6-99b9-72a827d5e6dc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D70B1C85-06A4-4402-967D-2C9EECE4E451}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB274801-13DF-4427-B402-2D080C779060}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5030cb7a-6be5-477a-957d-975e4d3028a7"/>
+    <ds:schemaRef ds:uri="83c7e37f-cb9c-4af6-99b9-72a827d5e6dc"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10446,12 +10553,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB274801-13DF-4427-B402-2D080C779060}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D70B1C85-06A4-4402-967D-2C9EECE4E451}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5030cb7a-6be5-477a-957d-975e4d3028a7"/>
-    <ds:schemaRef ds:uri="83c7e37f-cb9c-4af6-99b9-72a827d5e6dc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>